<commit_message>
change PR_AUC to key metric, Add augmentations to FlightDataset, TimeSeriesTransformer with mask
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,16 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://smu-my.sharepoint.com/personal/kh_nguyen_2025_mitb_smu_edu_sg/Documents/Data_Science/SMU/Study/Term 2/CS610 Applied ML/Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="8_{95C4CE0D-2520-4E0B-A98D-599385999CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77CD6F80-6976-469B-986F-FAEA47A2BC10}"/>
+  <xr:revisionPtr revIDLastSave="125" documentId="8_{95C4CE0D-2520-4E0B-A98D-599385999CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F912FBE-869D-4024-9B4E-B0BA6F4C71FB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3AEB3263-0B0E-46D1-87D0-7CDB5ACB019C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{3AEB3263-0B0E-46D1-87D0-7CDB5ACB019C}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="2" r:id="rId1"/>
     <sheet name="Experiments_full (2)" sheetId="4" r:id="rId2"/>
     <sheet name="Experiments_full" sheetId="3" r:id="rId3"/>
-    <sheet name="Experiments" sheetId="1" r:id="rId4"/>
+    <sheet name="Experiments (subset)" sheetId="1" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Experiments (subset)'!$A$1:$M$5</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -42,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="32">
   <si>
     <t>D_MODEL</t>
   </si>
@@ -223,14 +226,40 @@
   <si>
     <t>ROC-AUC</t>
   </si>
+  <si>
+    <t>PR-AUC</t>
+  </si>
+  <si>
+    <t>N_EPOCHS</t>
+  </si>
+  <si>
+    <t>DIM_FEEDFORWARD</t>
+  </si>
+  <si>
+    <t>Ex3</t>
+  </si>
+  <si>
+    <t>Recall(fail)</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>Acc</t>
+  </si>
+  <si>
+    <t>NUM_LAYERS</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="171" formatCode="0E+00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -285,7 +314,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -304,6 +333,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -470,22 +505,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>556260</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>1458</xdr:rowOff>
+      <xdr:colOff>541020</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>76162</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>488117</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>844348</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>64339</xdr:rowOff>
+      <xdr:rowOff>33801</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F7BFE7B8-51D4-FF48-471A-8160D4252F5A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{038A447C-32CB-3A79-8D43-E6226FE837B5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -501,8 +536,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="556260" y="1647378"/>
-          <a:ext cx="7689017" cy="2257441"/>
+          <a:off x="541020" y="1539202"/>
+          <a:ext cx="7039408" cy="2335079"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -514,22 +549,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>60960</xdr:colOff>
+      <xdr:colOff>1</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>106680</xdr:rowOff>
+      <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>336765</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>64349</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>106681</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>167179</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="5" name="Picture 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E6AD7F34-355F-D9C6-EEBE-A2345DB1AD72}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0990A35-AA16-0616-7931-7C72C888DEB5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -545,8 +580,52 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="670560" y="4130040"/>
-          <a:ext cx="7423365" cy="2152229"/>
+          <a:off x="609601" y="4023361"/>
+          <a:ext cx="7094220" cy="1081578"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7621</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>173382</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>155531</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27972AF1-6C0B-FF21-3B3A-9B5B45473D78}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="617221" y="5294022"/>
+          <a:ext cx="7208519" cy="3273989"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1287,15 +1366,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E2361BB-17A0-4C3F-9B6A-2513337F59A8}">
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="8" max="8" width="15.5546875" customWidth="1"/>
+    <col min="5" max="5" width="12.5546875" customWidth="1"/>
+    <col min="8" max="8" width="18.44140625" customWidth="1"/>
     <col min="9" max="9" width="13.88671875" customWidth="1"/>
     <col min="10" max="10" width="12.5546875" customWidth="1"/>
+    <col min="11" max="11" width="12.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -1309,28 +1390,34 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M1" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1340,32 +1427,32 @@
       <c r="C2" s="2">
         <v>64</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="8">
         <v>1E-3</v>
       </c>
-      <c r="E2" s="2">
-        <v>2</v>
+      <c r="E2" s="7">
+        <v>5</v>
       </c>
       <c r="F2" s="2">
+        <v>4</v>
+      </c>
+      <c r="G2" s="2">
         <v>0.1</v>
       </c>
-      <c r="G2" s="2">
-        <v>0.5</v>
-      </c>
       <c r="H2" s="2">
-        <v>0.4667</v>
-      </c>
-      <c r="I2" s="2">
-        <v>0.71050000000000002</v>
-      </c>
+        <v>512</v>
+      </c>
+      <c r="I2" s="2"/>
       <c r="J2" s="2">
-        <v>0.55879999999999996</v>
-      </c>
-      <c r="K2" s="2">
-        <v>0.63739999999999997</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+        <v>0.34549999999999997</v>
+      </c>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2">
+        <v>0.51190000000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1375,32 +1462,32 @@
       <c r="C3" s="2">
         <v>128</v>
       </c>
-      <c r="D3" s="3">
-        <v>1E-3</v>
-      </c>
-      <c r="E3" s="2">
-        <v>3</v>
+      <c r="D3" s="8">
+        <v>3.0000000000000001E-5</v>
+      </c>
+      <c r="E3" s="7">
+        <v>10</v>
       </c>
       <c r="F3" s="2">
+        <v>4</v>
+      </c>
+      <c r="G3" s="2">
         <v>0.1</v>
       </c>
-      <c r="G3" s="2">
-        <v>0.54169999999999996</v>
-      </c>
       <c r="H3" s="2">
-        <v>0.37719999999999998</v>
-      </c>
-      <c r="I3" s="2">
-        <v>1</v>
-      </c>
+        <v>512</v>
+      </c>
+      <c r="I3" s="2"/>
       <c r="J3" s="2">
-        <v>0.56889999999999996</v>
-      </c>
-      <c r="K3" s="2">
-        <v>0.81320000000000003</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+        <v>0.59340000000000004</v>
+      </c>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2">
+        <v>0.57250000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1408,22 +1495,40 @@
         <v>500</v>
       </c>
       <c r="C4" s="2">
-        <v>64</v>
-      </c>
-      <c r="D4" s="3">
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="E4" s="2">
-        <v>2</v>
+        <v>128</v>
+      </c>
+      <c r="D4" s="8">
+        <v>1E-4</v>
+      </c>
+      <c r="E4" s="7">
+        <v>15</v>
       </c>
       <c r="F4" s="2">
-        <v>0.1</v>
-      </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="H4" s="2">
+        <v>512</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0.66669999999999996</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0.66010000000000002</v>
+      </c>
+      <c r="K4" s="2">
+        <v>0.76319999999999999</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0.72060000000000002</v>
+      </c>
+      <c r="M4">
+        <v>0.66590000000000005</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1431,22 +1536,40 @@
         <v>500</v>
       </c>
       <c r="C5" s="2">
-        <v>64</v>
-      </c>
-      <c r="D5" s="3">
-        <v>1E-3</v>
-      </c>
-      <c r="E5" s="2">
-        <v>2</v>
+        <v>256</v>
+      </c>
+      <c r="D5" s="8">
+        <v>1E-4</v>
+      </c>
+      <c r="E5" s="7">
+        <v>10</v>
       </c>
       <c r="F5" s="2">
-        <v>0.3</v>
-      </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H5" s="2">
+        <v>1024</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0.69440000000000002</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0.69350000000000001</v>
+      </c>
+      <c r="K5" s="2">
+        <v>0.60529999999999995</v>
+      </c>
+      <c r="L5" s="2">
+        <v>0.73680000000000001</v>
+      </c>
+      <c r="M5">
+        <v>0.73119999999999996</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1456,7 +1579,13 @@
         <v>21</v>
       </c>
     </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:M5" xr:uid="{5E2361BB-17A0-4C3F-9B6A-2513337F59A8}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>